<commit_message>
English only; neutral wording for AI assistance; BOM candidate rows in English
</commit_message>
<xml_diff>
--- a/bom/bom.xlsx
+++ b/bom/bom.xlsx
@@ -729,7 +729,7 @@
     <row r="4" hidden="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>[ALT qty0] SKF PCM 121420 E - bushing radente PTFE composito 12x14x20 mm</t>
+          <t>[ALT qty0] SKF PCM 121420 E - PTFE composite plain bushing 12x14x20 mm</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -762,12 +762,12 @@
       <c r="M4" s="4" t="n"/>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>Esempio reale di bushing radente sottile per un axis diametro 12 mm del giunto foot-shin: bore 12 mm, esterno 14 mm, lunghezza 20 mm.</t>
+          <t>Real example of a thin plain bushing for a 12 mm diameter shaft of the foot-shin joint: bore 12 mm, outer diameter 14 mm, length 20 mm.</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU SKF PCM121420E. Price checked 2026-06-02: EUR 2.13 netto. Alternative candidata per oscillazione lenta; qty 0 finche CAD, carichi, accoppiamento pin-sede and control assiale non sono definiti.</t>
+          <t>Exact SKU SKF PCM121420E. Price verified 2026-06-02: EUR 2.13 net (excluding VAT). Candidate alternative for slow oscillation; qty 0 until CAD, loads, pin-seat fit and axial control are defined.</t>
         </is>
       </c>
       <c r="P4" s="4" t="inlineStr">
@@ -791,7 +791,7 @@
     <row r="5" hidden="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>[ALT qty0] SKF PCM 121425 E - bushing radente PTFE composito 12x14x25 mm</t>
+          <t>[ALT qty0] SKF PCM 121425 E - PTFE composite plain bushing 12x14x25 mm</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -824,12 +824,12 @@
       <c r="M5" s="4" t="n"/>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>Esempio reale piu lungo della stessa famiglia: bore 12 mm, esterno 14 mm, lunghezza 25 mm. Dimostra che una bushing unica lunga 25 mm and un componente standard.</t>
+          <t>Longer real example from the same family: bore 12 mm, outer diameter 14 mm, length 25 mm. It shows that a single 25 mm long bushing is a standard component.</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU SKF PCM121425E. Price checked 2026-06-02: EUR 2.94 netto. Qty 0: la maggiore lunghezza non and automaticamente migliore se introduce disallineamento o se il CAD non offre una sede corretta.</t>
+          <t>Exact SKU SKF PCM121425E. Price verified 2026-06-02: EUR 2.94 net (excluding VAT). Qty 0: the greater length is not automatically better if it introduces misalignment or if the CAD does not provide a correct seat.</t>
         </is>
       </c>
       <c r="P5" s="4" t="inlineStr">
@@ -853,7 +853,7 @@
     <row r="6" hidden="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>[ALT qty0] igus iglidur Q2SM-1214-20 - bushing polimerica heavy-duty 12x14x20 mm</t>
+          <t>[ALT qty0] igus iglidur Q2SM-1214-20 - heavy-duty polymer bushing 12x14x20 mm</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -886,12 +886,12 @@
       <c r="M6" s="4" t="n"/>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>Esempio polimerico autolubrificante per axis diametro 12 mm: esterno 14 mm, lunghezza 20 mm. Il materiale Q2 and sviluppato per applicazioni pivotanti with carichi dinamici, urti and sporco.</t>
+          <t>Self-lubricating polymer example for a 12 mm diameter shaft: outer diameter 14 mm, length 20 mm. The Q2 material is developed for pivoting applications with dynamic loads, shocks and dirt.</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU igus Q2SM-1214-20. Price checked 2026-06-02: PLN 25.89 netto, about EUR 6.15. Qty 0: check pressione superficiale, usura, sede and tolleranze with il tool igus prima della selezione.</t>
+          <t>Exact SKU igus Q2SM-1214-20. Price verified 2026-06-02: PLN 25.89 net (excluding VAT), about EUR 6.15. Qty 0: verify surface pressure, wear, seat and tolerances with the igus tool before selection.</t>
         </is>
       </c>
       <c r="P6" s="4" t="inlineStr">
@@ -915,7 +915,7 @@
     <row r="7" hidden="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>[ALT qty0] igus iglidur Q2FM-1214-12 - bushing flangiata heavy-duty 12x14x12 mm</t>
+          <t>[ALT qty0] igus iglidur Q2FM-1214-12 - heavy-duty flanged bushing 12x14x12 mm</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -948,12 +948,12 @@
       <c r="M7" s="4" t="n"/>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>Esempio di bushing radente flangiata per pin diametro 12 mm: guida il carico radiale and offre una battuta assiale integrata. Dimensions: bore 12 mm, esterno 14 mm, lunghezza 12 mm, flangia diametro 20 mm spessa 1 mm.</t>
+          <t>Example of a flanged plain bushing for a 12 mm diameter pin: it guides the radial load and provides an integrated axial stop. Dimensions: bore 12 mm, outer diameter 14 mm, length 12 mm, flange diameter 20 mm, 1 mm thick.</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU igus Q2FM-1214-12. Qty 0: utile se il CAD permette una bushing inserita da ciascun lato del pezzo mobile; non assumere che due pcs da 12 mm entrino nella larghezza disponibile. Q2 and indicato da igus per carichi elevati, urti, sporco and applicazioni pivotanti fortemente sollecitate.</t>
+          <t>Exact SKU igus Q2FM-1214-12. Qty 0: useful if the CAD allows one bushing inserted from each side of the moving part; do not assume that two 12 mm pieces fit in the available width. Q2 is indicated by igus for high loads, shocks, dirt and heavily stressed pivoting applications.</t>
         </is>
       </c>
       <c r="P7" s="4" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="8" hidden="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>[ARCHIVED qty0] igus GTM-1224-015 - ralla separata (superata: assiale ora nella flangia) 12x24x1.5 mm</t>
+          <t>[ARCHIVED qty0] igus GTM-1224-015 - separate thrust washer (superseded: axial now in the flange) 12x24x1.5 mm</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1010,12 +1010,12 @@
       <c r="M8" s="4" t="n"/>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>Ralla radente separata da registrare sul pezzo centrale mobile tra questo and ciascuna orecchia esterna quando la bushing radiale non ha flangia. Porta lo strisciamento assiale su una superficie progettata allo scopo.</t>
+          <t>Separate plain thrust washer to be located on the central moving part, between it and each outer lug, when the radial bushing has no flange. It puts the axial sliding on a surface designed for the purpose.</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU igus GTM-1224-015: bore 12 mm, esterno 24 mm, spessore 1.5 mm. Price checked 2026-06-02: EUR 1.49 IVA inclusa su Conrad. Qty 0: non lasciarla libera tra due facce PA-CF. Prevedere una sede di registrazione and una controfaccia metallica fissa, liscia and sostituibile nell'orecchia; definire gioco assiale nel CAD.</t>
+          <t>Exact SKU igus GTM-1224-015: bore 12 mm, outer diameter 24 mm, thickness 1.5 mm. Price verified 2026-06-02: EUR 1.49 VAT included at Conrad. Qty 0: do not leave it loose between two PA-CF faces. Provide a locating seat and a fixed, smooth, replaceable metal counterface in the lug; define the axial play in the CAD.</t>
         </is>
       </c>
       <c r="P8" s="4" t="inlineStr">
@@ -1039,7 +1039,7 @@
     <row r="9" hidden="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>[ARCHIVED qty0] SKF HK 1216.2RS - rullini without anello interno (superato) 12x18x16 mm</t>
+          <t>[ARCHIVED qty0] SKF HK 1216.2RS - needle roller bearing without inner ring (superseded) 12x18x16 mm</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1072,12 +1072,12 @@
       <c r="M9" s="4" t="n"/>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>Alternative volvente compatta per il solo carico radiale del pin diametro 12 mm. Va alloggiata nel pezzo mobile oppure nella coppia di orecchie, non contemporaneamente in entrambi. Non possiede un anello interno da serrare tra gli spallamenti delle orecchie.</t>
+          <t>Compact rolling alternative for the radial load only of the 12 mm diameter pin. It must be housed either in the moving part or in the pair of lugs, not in both at the same time. It has no inner ring to clamp between the shoulders of the lugs.</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU SKF HK1216.2RS: bore 12 mm, esterno 18 mm, lunghezza 16 mm, tenute su entrambi i lati. Disponibilita verificata 2026-06-02: 21 pcs, prezzo su quotazione. Qty 0: richiede che il pin fisso sia una pista interna temprata and rettificata adeguata; non far lavorare automaticamente i rullini su una vite o un pin grezzo. Non and la prima scelta se si vogliono serrare spallamenti contro un vero anello interno.</t>
+          <t>Exact SKU SKF HK1216.2RS: bore 12 mm, outer diameter 18 mm, length 16 mm, seals on both sides. Availability verified 2026-06-02: 21 pieces, price on quotation. Qty 0: it requires the fixed pin to be a suitable hardened and ground inner raceway; do not automatically let the needle rollers run on a screw or a raw pin. It is not the first choice if you want to clamp shoulders against a true inner ring.</t>
         </is>
       </c>
       <c r="P9" s="4" t="inlineStr">
@@ -1101,7 +1101,7 @@
     <row r="10" hidden="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>[ARCHIVED qty0] SKF NKI 12/16 - rullini with anello interno (superato dal radente igus flangiato) 12x24x16 mm</t>
+          <t>[ARCHIVED qty0] SKF NKI 12/16 - needle roller bearing with inner ring (superseded by the flanged igus plain bushing) 12x24x16 mm</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -1134,12 +1134,12 @@
       <c r="M10" s="4" t="n"/>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>Prima architettura semplice da disegnare: bearing nel pezzo centrale mobile; anello interno separabile serrato tra gli spallamenti integrati delle due orecchie PA-CF; anello esterno in sede nel centro mobile. Porta il carico radiale without richiedere cappelli metallici nelle orecchie.</t>
+          <t>First simple architecture to draw: bearing in the central moving part; separable inner ring clamped between the integrated shoulders of the two PA-CF lugs; outer ring seated in the moving centre. It carries the radial load without requiring metal caps in the lugs.</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU SKF NKI 12/16: bore 12 mm, esterno 24 mm, larghezza 16 mm, anello interno incluso. Price checked 2026-06-02: EUR 22.15 netto su Klium. Qty 0 fino al CAD. Gli spallamenti devono serrare l'anello interno without schiacciare il pezzo centrale mobile; il gioco di funzionamento and tra parte mobile and orecchie, non tra spallamenti and anello interno. NKI non and un reggispinta: se i test mostrano contatto assiale, aggiungere ralle igus registrate oppure un reggispinta separato.</t>
+          <t>Exact SKU SKF NKI 12/16: bore 12 mm, outer diameter 24 mm, width 16 mm, inner ring included. Price verified 2026-06-02: EUR 22.15 net (excluding VAT) at Klium. Qty 0 until the CAD. The shoulders must clamp the inner ring without crushing the central moving part; the running clearance is between the moving part and the lugs, not between the shoulders and the inner ring. NKI is not a thrust bearing: if tests show axial contact, add located igus thrust washers or a separate thrust bearing.</t>
         </is>
       </c>
       <c r="P10" s="4" t="inlineStr">
@@ -1163,7 +1163,7 @@
     <row r="11" hidden="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>[ARCHIVED qty0] SKF AXK 1226 - reggispinta (superato: assiale ora nella flangia) 12x26x2 mm</t>
+          <t>[ARCHIVED qty0] SKF AXK 1226 - thrust bearing (superseded: axial now in the flange) 12x26x2 mm</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1196,12 +1196,12 @@
       <c r="M11" s="4" t="n"/>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>Alternative volvente per carico assiale: una gabbia reggispinta per ciascun lato del pezzo centrale mobile se il CAD richiede attrito assiale molto ridotto.</t>
+          <t>Rolling alternative for axial load: one thrust bearing cage for each side of the central moving part if the CAD requires very low axial friction.</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU SKF AXK 1226: bore 12 mm, esterno 26 mm, spessore 2 mm, carico dinamico 9.15 kN and statico 30 kN. Price checked 2026-06-02: EUR 4.10 netto su RS Italia. Qty 0: tra facce stampate usare due ralle temprate AS 1226 per ciascuna gabbia.</t>
+          <t>Exact SKU SKF AXK 1226: bore 12 mm, outer diameter 26 mm, thickness 2 mm, dynamic load 9.15 kN and static 30 kN. Price verified 2026-06-02: EUR 4.10 net (excluding VAT) at RS Italia. Qty 0: between printed faces use two hardened AS 1226 washers for each cage.</t>
         </is>
       </c>
       <c r="P11" s="4" t="inlineStr">
@@ -1225,7 +1225,7 @@
     <row r="12" hidden="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>[ARCHIVED qty0] SKF AS 1226 - ralla temprata per AXK (superato) 12x26x1 mm</t>
+          <t>[ARCHIVED qty0] SKF AS 1226 - hardened thrust washer for AXK (superseded) 12x26x1 mm</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1258,12 +1258,12 @@
       <c r="M12" s="4" t="n"/>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>Pista assiale temprata per la gabbia AXK 1226. Con facce PA-CF o polimeriche non usare direttamente il pezzo stampato come pista dei rullini.</t>
+          <t>Hardened axial raceway for the AXK 1226 cage. With PA-CF or polymer faces do not use the printed part directly as the raceway for the needle rollers.</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU SKF AS1226: bore 12 mm, esterno 26 mm, spessore 1 mm. Prezzo and stock verificati 2026-06-02: EUR 1.86 netto, 13 pcs disponibili. Qty 0: una soluzione completa per lato occupa 1 + 2 + 1 = 4 mm: AS 1226 + AXK 1226 + AS 1226.</t>
+          <t>Exact SKU SKF AS1226: bore 12 mm, outer diameter 26 mm, thickness 1 mm. Price and stock verified 2026-06-02: EUR 1.86 net (excluding VAT), 13 pieces available. Qty 0: a complete solution per side takes up 1 + 2 + 1 = 4 mm: AS 1226 + AXK 1226 + AS 1226.</t>
         </is>
       </c>
       <c r="P12" s="4" t="inlineStr">
@@ -1287,7 +1287,7 @@
     <row r="13" hidden="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">[ARCHIVED qty0] HGI PS 12x18x1 DIN 988 - rasamento di registro (superato) </t>
+          <t xml:space="preserve">[ARCHIVED qty0] HGI PS 12x18x1 DIN 988 - adjustment shim washer (superseded) </t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1320,12 +1320,12 @@
       <c r="M13" s="4" t="n"/>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>Rasamento metallico per calibrare il gioco assiale residuo dopo aver selected la superficie reggispinta. Non sostituisce una ralla radente igus o una pista temprata per AXK.</t>
+          <t>Metal shim washer to calibrate the residual axial play after choosing the thrust surface. It does not replace an igus plain thrust washer or a hardened raceway for AXK.</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU HGI12X18X1 / PS12X18X1: bore 12 mm, esterno 18 mm, spessore 1 mm. Prezzo and stock verificati 2026-06-02: EUR 0.48 netto, 57 pcs. Qty 0: scegliere la combinazione finale solo dopo misura dell'assieme; DIN 988 esiste anche in spessori piu fini, ad esempio 0.2 mm.</t>
+          <t>Exact SKU HGI12X18X1 / PS12X18X1: bore 12 mm, outer diameter 18 mm, thickness 1 mm. Price and stock verified 2026-06-02: EUR 0.48 net (excluding VAT), 57 pieces. Qty 0: choose the final combination only after measuring the assembly; DIN 988 also exists in finer thicknesses, for example 0.2 mm.</t>
         </is>
       </c>
       <c r="P13" s="4" t="inlineStr">
@@ -1349,7 +1349,7 @@
     <row r="14" hidden="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>[ALT TO SIZE qty0] Inserti metallici flangiati fissi nelle orecchie ankle - controfacce per axis diam. 12 mm</t>
+          <t>[ALT TO SIZE qty0] Fixed flanged metal inserts in the ankle lugs - counterfaces for 12 mm diam. axis</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1382,12 +1382,12 @@
       <c r="M14" s="4" t="n"/>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>Due inserti a cappello per axis, pressati o registrati nelle orecchie esterne PA-CF: il bore interno guida o contiene il pin fisso diametro 12 mm; la flangia rivolta verso il pezzo centrale offre una controfaccia assiale metallica liscia alla ralla igus.</t>
+          <t>Two cap-shaped inserts per axis, pressed or located in the outer PA-CF lugs: the inner bore guides or contains the fixed 12 mm diameter pin; the flange facing the central part provides a smooth metal axial counterface for the igus thrust washer.</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>Alternative da tenere documentata se si usa la bushing igus centrale stampata oppure se gli spallamenti PA-CF non risultano sufficienti. Reference preliminare CAD: orecchio sinistro about 20 mm + pezzo centrale mobile with bushing about 20 mm + orecchio destro about 20 mm = about 60 mm di corpi strutturali. I cappelli vanno su entrambe le orecchie. Attenzione: una flangia sporgente aumenta il pacco; incassarla nell'orecchia se si vuole restare vicini ai 60 mm. Il bore del cappello guida il pin ma non lo rende automaticamente solidale alle orecchie: progettare anche antirotazione and ritegno assiale.</t>
+          <t>Alternative to keep documented if the printed central igus bushing is used or if the PA-CF shoulders prove insufficient. Preliminary CAD reference: left lug about 20 mm + central moving part with bushing about 20 mm + right lug about 20 mm = about 60 mm of structural bodies. The caps go on both lugs. Caution: a protruding flange increases the stack; recess it into the lug if you want to stay close to 60 mm. The cap bore guides the pin but does not automatically make it integral with the lugs: also design anti-rotation and axial retention.</t>
         </is>
       </c>
       <c r="P14" s="4" t="inlineStr">
@@ -1411,7 +1411,7 @@
     <row r="15" hidden="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>[OPTIONAL UPGRADE qty0] Elesa+Ganter GN.12825 / DIN 172-B12-20-A - controfaccia metallica nell'orecchia, bore 12 L20</t>
+          <t>[OPTIONAL UPGRADE qty0] Elesa+Ganter GN.12825 / DIN 172-B12-20-A - metal counterface in the lug, bore 12 L20</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1444,12 +1444,12 @@
       <c r="M15" s="4" t="n"/>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>Candidato standard per ciascuna orecchia se si stampa la bushing centrale igus: bussola guida temprata a cappello, bore interno 12 mm F7, esterno 18 mm n6, flangia diametro 22 mm, corpo lungo 20 mm and flangia spessa 4 mm.</t>
+          <t>Standard candidate for each lug if the central igus bushing is printed: hardened cap-type guide bush, inner bore 12 mm F7, outer diameter 18 mm n6, flange diameter 22 mm, body 20 mm long and flange 4 mm thick.</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU Elesa+Ganter DIN172-B12-20-A / GN.12825, codice Verzolla Y1137. Prezzo and disponibilita verificati 2026-06-02: EUR 6.89 each, 5 disponibili. Qty 0: quantity attesa se usata su entrambi gli assi and su entrambe le caviglie = 8 pcs, ma attivare solo dopo CAD. Per mantenere il reference about 60 mm incassare la flangia da 4 mm nell'orecchia; check inoltre controfaccia, fit nel PA-CF and antirotazione del pin.</t>
+          <t>Exact SKU Elesa+Ganter DIN172-B12-20-A / GN.12825, Verzolla code Y1137. Price and availability verified 2026-06-02: EUR 6.89 each, 5 available. Qty 0: expected quantity if used on both axes and on both ankles = 8 pieces, but activate only after CAD. To keep the about 60 mm reference, recess the 4 mm flange into the lug; also verify counterface, fit in the PA-CF and anti-rotation of the pin.</t>
         </is>
       </c>
       <c r="P15" s="4" t="inlineStr">
@@ -1473,7 +1473,7 @@
     <row r="16" hidden="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>[ALT FORNITORE qty0] Otto Ganter 172-B12-20-A - cappello metallico flangiato bore 12 mm, L20</t>
+          <t>[ALT SUPPLIER qty0] Otto Ganter 172-B12-20-A - flanged metal cap, bore 12 mm, L20</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1506,12 +1506,12 @@
       <c r="M16" s="4" t="n"/>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>Secondo fornitore dello stesso cappello normalizzato DIN 172-B12-20-A: acciaio, bore 12 mm, esterno 18 mm, flangia 22 mm, lunghezza corpo 20 mm, flangia 4 mm.</t>
+          <t>Second supplier of the same standardized DIN 172-B12-20-A cap: steel, bore 12 mm, outer diameter 18 mm, flange 22 mm, body length 20 mm, flange 4 mm.</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>Exact product Ganter 172-B12-20-A. Prezzo and consegna verificati 2026-06-02: EUR 5.26 netto each, indicato spedibile in 2-3 giorni lavorativi; vendita B2B. Qty 0: alternative di approvvigionamento allo stesso componente Verzolla.</t>
+          <t>Exact product Ganter 172-B12-20-A. Price and delivery verified 2026-06-02: EUR 5.26 net (excluding VAT) each, indicated as shippable in 2-3 working days; B2B sales. Qty 0: sourcing alternative for the same Verzolla component.</t>
         </is>
       </c>
       <c r="P16" s="4" t="inlineStr">
@@ -1535,7 +1535,7 @@
     <row r="17" hidden="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>[ALT EQUIVALENTE qty0] KIPP K1022.A1200X20 - cappello metallico flangiato DIN 172 bore 12 mm, L20</t>
+          <t>[ALT EQUIVALENT qty0] KIPP K1022.A1200X20 - flanged metal cap DIN 172, bore 12 mm, L20</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1568,12 +1568,12 @@
       <c r="M17" s="4" t="n"/>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>Equivalente DIN 172 forma A di altro produttore per lo stesso dimensionamento preliminare: bussola a cappello in acciaio with bore interno 12 mm and lunghezza 20 mm.</t>
+          <t>DIN 172 form A equivalent from another manufacturer for the same preliminary sizing: steel cap-type bush with inner bore 12 mm and length 20 mm.</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU KIPP K1022.A1200X20. Prezzo and disponibilita verificati 2026-06-02: EUR 4.50 netto / EUR 5.36 IVA inclusa each, indicato disponibile with consegna 2-5 giorni. Qty 0: alternative standard da check dimensionalmente contro il disegno KIPP prima dell'ordine.</t>
+          <t>Exact SKU KIPP K1022.A1200X20. Price and availability verified 2026-06-02: EUR 4.50 net (excluding VAT) / EUR 5.36 VAT included each, indicated as available with delivery in 2-5 days. Qty 0: standard alternative to be verified dimensionally against the KIPP drawing before ordering.</t>
         </is>
       </c>
       <c r="P17" s="4" t="inlineStr">
@@ -1597,7 +1597,7 @@
     <row r="18" hidden="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>[SCHEDA qty0] Elesa+Ganter DIN 172-B12-20-A - pagina tecnica TME</t>
+          <t>[DATASHEET qty0] Elesa+Ganter DIN 172-B12-20-A - TME technical page</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1630,12 +1630,12 @@
       <c r="M18" s="4" t="n"/>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t>Pagina tecnica di un ulteriore distributore per lo stesso cappello Ganter: acciaio temprato, bore interno 12 mm, esterno 18 mm, flangia 22 mm, lunghezza 20 mm.</t>
+          <t>Technical page of a further distributor for the same Ganter cap: hardened steel, inner bore 12 mm, outer diameter 18 mm, flange 22 mm, length 20 mm.</t>
         </is>
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU TME DIN172-B12-20-A. Verificato 2026-06-02: USD 10.04 about EUR 9.27 each, ma stock TME indicato zero. Tenerlo come catalogo tecnico and backup di richiesta disponibilita, non come fornitore primario immediato.</t>
+          <t>Exact SKU TME DIN172-B12-20-A. Verified 2026-06-02: USD 10.04 about EUR 9.27 each, but TME stock indicated as zero. Keep it as a technical catalogue and as a backup for availability requests, not as an immediate primary supplier.</t>
         </is>
       </c>
       <c r="P18" s="4" t="inlineStr">
@@ -1659,7 +1659,7 @@
     <row r="19" hidden="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>[ALT CUSTOM qty0] Bushing radente stampata 3D in igus iglidur i150</t>
+          <t>[ALT CUSTOM qty0] 3D printed plain bushing in igus iglidur i150</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1692,12 +1692,12 @@
       <c r="M19" s="4" t="n"/>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>Primo provino custom stampabile per gli assi diametro 12 mm del giunto foot-shin. Permette di iterare lunghezza, flangia and gioco. i150 and il tribofilamento igus piu facile da processare.</t>
+          <t>First printable custom test piece for the 12 mm diameter axes of the foot-shin joint. It allows iterating on length, flange and play. i150 is the easiest igus tribofilament to process.</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>Materiale confermato tra quelli che l'utente sta acquistando per confronto. Qty 0: non and ancora la scelta finale. Validare pressione superficiale, usura, orientamento di stampa, finitura del pin, tolleranze and gioco; non assumere automaticamente equivalenza with Q2 stampato a iniezione o SKF metallo/PTFE.</t>
+          <t>Material confirmed among those the user is purchasing for comparison. Qty 0: it is not yet the final choice. Validate surface pressure, wear, print orientation, pin finish, tolerances and play; do not automatically assume equivalence with injection-moulded Q2 or SKF metal/PTFE.</t>
         </is>
       </c>
       <c r="P19" s="4" t="inlineStr">
@@ -1721,7 +1721,7 @@
     <row r="20" hidden="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>[ALT CUSTOM qty0] Bushing radente stampata 3D in igus iglidur i190</t>
+          <t>[ALT CUSTOM qty0] 3D printed plain bushing in igus iglidur i190</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1754,12 +1754,12 @@
       <c r="M20" s="4" t="n"/>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t>Secondo provino custom stampabile per gli assi diametro 12 mm del giunto foot-shin. i190 and il candidato da confrontare quando servono maggiore resistenza meccanica and resistenza all'usura.</t>
+          <t>Second printable custom test piece for the 12 mm diameter axes of the foot-shin joint. i190 is the candidate to compare when greater mechanical strength and wear resistance are needed.</t>
         </is>
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>Materiale confermato tra quelli che l'utente sta acquistando per confronto. Qty 0: non and ancora la scelta finale. Il filamento and sensibile all'umidita: seguire essiccazione and istruzioni igus. Validare pressione superficiale, usura, orientamento, tolleranze and gioco.</t>
+          <t>Material confirmed among those the user is purchasing for comparison. Qty 0: it is not yet the final choice. The filament is sensitive to moisture: follow igus drying and instructions. Validate surface pressure, wear, orientation, tolerances and play.</t>
         </is>
       </c>
       <c r="P20" s="4" t="inlineStr">
@@ -1783,7 +1783,7 @@
     <row r="21" hidden="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>[SELECTED PRIMARIO qty0] Bushing STAMPATA multimateriale J260+PA-CF integrale (radiale + flangia assiale)</t>
+          <t>[CHOSEN PRIMARY qty0] PRINTED multi-material bushing J260+PA-CF, integral (radial + axial flange)</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1816,12 +1816,12 @@
       <c r="M21" s="4" t="n"/>
       <c r="N21" s="3" t="inlineStr">
         <is>
-          <t>Approccio PRIMARIO selected: stampare la bushing direttamente integrale al pezzo mobile PA-CF in FDM multimateriale, with J260 sia sul bore (radiale) sia sulle facce di flangia (assiale). Nessun acquisto se la stampa regge.</t>
+          <t>PRIMARY approach chosen: print the bushing directly integral with the PA-CF moving part in multi-material FDM, with J260 both on the bore (radial) and on the flange faces (axial). No purchase if the print holds up.</t>
         </is>
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>Filamento J260-PF gia acquistato dall'utente. igus indica estrusione ~280 C, piano ~120 C, preferibile camera riscaldata. To validate in modo specifico: adesione all'interfaccia J260/PA-CF (rischio principale del multimateriale), orientamento di stampa per roundness and usura del bore, finitura and Ø reale (prevedere alesatura/taratura), pressione superficiale, gioco. Qty 0: gestita dal filamento, non da uno SKU. i150 and i190 restano provini di confronto.</t>
+          <t>J260-PF filament already purchased by the user. igus indicates extrusion ~280 C, bed ~120 C, heated chamber preferable. To be validated specifically: adhesion at the J260/PA-CF interface (main risk of multi-material), print orientation for roundness and bore wear, finish and actual Ø (plan for reaming/calibration), surface pressure, play. Qty 0: handled by the filament, not by an SKU. i150 and i190 remain comparison test pieces.</t>
         </is>
       </c>
       <c r="P21" s="4" t="inlineStr">
@@ -1845,7 +1845,7 @@
     <row r="22" hidden="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>[SELECTED FALLBACK qty0] Bushing flangiata igus GFM-1214 (iglidur G) - radiale + assiale, acquistabile</t>
+          <t>[CHOSEN FALLBACK qty0] igus GFM-1214 flanged bushing (iglidur G) - radial + axial, purchasable</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -1878,12 +1878,12 @@
       <c r="M22" s="4" t="n"/>
       <c r="N22" s="3" t="inlineStr">
         <is>
-          <t>Versione ACQUISTATA della bushing flangiata, fallback se la stampa multimateriale J260 non regge: bore 12, esterno 14, flangia about 20 x 1. La flangia fa l'assiale; due per axis, flange verso l'esterno, piantate a pressione nel pezzo mobile. Drop-in stesse quote: Q2FM-1214 (heavy-duty urti/sporco), JFM-1214 (basso attrito).</t>
+          <t>PURCHASED version of the flanged bushing, fallback if the J260 multi-material print does not hold up: bore 12, outer diameter 14, flange about 20 x 1. The flange handles the axial load; two per axis, flanges facing outwards, press-fitted into the moving part. Drop-in with the same dimensions: Q2FM-1214 (heavy-duty shocks/dirt), JFM-1214 (low friction).</t>
         </is>
       </c>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>Famiglia SKU GFM-1214 iglidur G. Lunghezza b1 dal CAD (es. due da 9-10 mm in un mobile da 20 mm). Fornitori multipli verificati 2026-06-03: igus diretto, RS, Misumi IT, Minetti, F.lli Bono, Solema, ERIKS. Qty 0 finche il CAD non da le lunghezze; quantity attesa 8 (2 per axis x 4 assi) solo se si comprano invece di stamparle. Ritegno: interferenza nella sede + flangia di battuta; mai cianoacrilato, al limite Loctite 603/638. Prezzo da check a configurazione lunghezza.</t>
+          <t>SKU family GFM-1214 iglidur G. Length b1 from the CAD (e.g. two of 9-10 mm in a 20 mm moving part). Multiple suppliers verified 2026-06-03: igus direct, RS, Misumi IT, Minetti, F.lli Bono, Solema, ERIKS. Qty 0 until the CAD gives the lengths; expected quantity 8 (2 per axis x 4 axes) only if they are bought instead of printed. Retention: interference in the seat + stop flange; never cyanoacrylate, at most Loctite 603/638. Price to be verified once the length is configured.</t>
         </is>
       </c>
       <c r="P22" s="4" t="inlineStr">
@@ -1969,7 +1969,7 @@
     <row r="24" hidden="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>[CATALOGO qty0] RS PRO 822-9316 - shoulder screw M10, spallamento diam. 12 x 20 mm</t>
+          <t>[CATALOGUE qty0] RS PRO 822-9316 - shoulder screw M10, shoulder diam. 12 x 20 mm</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -2002,12 +2002,12 @@
       <c r="M24" s="4" t="n"/>
       <c r="N24" s="3" t="inlineStr">
         <is>
-          <t>Esempio industriale acquistabile di vite a spallamento: filetto M10, diametro spallamento 12 mm, lunghezza spallamento 20 mm, acciaio nero classe 12.9.</t>
+          <t>Purchasable industrial example of a shoulder screw: M10 thread, shoulder diameter 12 mm, shoulder length 20 mm, black steel class 12.9.</t>
         </is>
       </c>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU RS PRO 822-9316. Price checked 2026-06-02: EUR 31.71 netto per sacchetto da quattro, EUR 7.928 each. Qty 0: la lunghezza 20 mm and solo un reference di catalogo; scegliere la lunghezza effettiva dopo il CAD.</t>
+          <t>Exact SKU RS PRO 822-9316. Price verified 2026-06-02: EUR 31.71 net (excluding VAT) per bag of four, EUR 7.928 each. Qty 0: the 20 mm length is only a catalogue reference; choose the actual length after the CAD.</t>
         </is>
       </c>
       <c r="P24" s="4" t="inlineStr">
@@ -2031,7 +2031,7 @@
     <row r="25" hidden="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>[ALT qty0] RS PRO 292-417 - shoulder screw ISO 7379 M10, gambo Ø12 x 60 mm (alternative industriale al nero AliExpress)</t>
+          <t>[ALT qty0] RS PRO 292-417 - shoulder screw ISO 7379 M10, shank Ø12 x 60 mm (industrial alternative to the black AliExpress one)</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -2064,12 +2064,12 @@
       <c r="M25" s="4" t="n"/>
       <c r="N25" s="3" t="inlineStr">
         <is>
-          <t>Reference vicino al primo pacco CAD ankle about 60 mm: vite ISO 7379 with tratto liscio diametro 12 mm lungo 60 mm, filetto M10 x 16 mm, testa diametro 18 x 8 mm, lunghezza totale 84 mm.</t>
+          <t>Reference close to the first ankle CAD stack of about 60 mm: ISO 7379 screw with a plain section of diameter 12 mm and length 60 mm, thread M10 x 16 mm, head diameter 18 x 8 mm, total length 84 mm.</t>
         </is>
       </c>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU RS PRO 292-417, ISO 7379 gambo Ø12 x 60, filetto M10 x 16, testa Ø18 x 8. ALTERNATIVA industriale (il pin selected e' ora la shoulder screw nera AliExpress Ø12xM10): fa da pista su cui scorre l'igus and da ritegno. Reso solidale alle orecchie dal serraggio (nut M10 + Loctite 243), non da piantaggio; fit gambo-bore orecchia scorrevole-bloccato (snug), no interferenza forte nel PA-CF. Expected qty 4 (un axis ciascuno) + scorte, ma qty 0 finche il CAD non fissa la lunghezza colletto (~60-70). Fornitori alternativi ISO 7379-12-M10: Rubix GN.35185, Elesa, Puntoviti, Berardi, KIPP.</t>
+          <t>Exact SKU RS PRO 292-417, ISO 7379 shank Ø12 x 60, thread M10 x 16, head Ø18 x 8. Industrial ALTERNATIVE (the chosen pin is now the black AliExpress shoulder screw Ø12xM10): it acts as the raceway on which the igus slides and as retention. Made integral with the lugs by clamping (M10 nut + Loctite 243), not by press-fitting; shank-to-lug-bore fit sliding-locked (snug), no strong interference in the PA-CF. Expected qty 4 (one axis each) + spares, but qty 0 until the CAD fixes the shoulder length (~60-70). Alternative suppliers ISO 7379-12-M10: Rubix GN.35185, Elesa, Puntoviti, Berardi, KIPP.</t>
         </is>
       </c>
       <c r="P25" s="4" t="inlineStr">
@@ -2093,7 +2093,7 @@
     <row r="26" hidden="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>[CATALOGO qty0] Motedis 12h6 - albero precisione diam. 12 mm h6 temprato and rettificato</t>
+          <t>[CATALOGUE qty0] Motedis 12h6 - precision shaft diam. 12 mm h6 hardened and ground</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -2126,12 +2126,12 @@
       <c r="M26" s="4" t="n"/>
       <c r="N26" s="3" t="inlineStr">
         <is>
-          <t>Alternative da tagliare a misura quando serve un pin fisso cilindrico without testa. Utile anche come pista temprata and rettificata se si valuta un bearing HK privo di anello interno.</t>
+          <t>Alternative to be cut to size when a headless cylindrical fixed pin is needed. Also useful as a hardened and ground raceway if an HK bearing without inner ring is being considered.</t>
         </is>
       </c>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>Codice prodotto Motedis 12h6. Qty 0: prezzo dipendente dalla lunghezza di taglio. Definire lunghezza and ritegno; non sostituisce automaticamente una vite a spallamento.</t>
+          <t>Motedis product code 12h6. Qty 0: price dependent on the cut length. Define length and retention; it does not automatically replace a shoulder screw.</t>
         </is>
       </c>
       <c r="P26" s="4" t="inlineStr">
@@ -2155,7 +2155,7 @@
     <row r="27" hidden="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>[CATALOGO qty0] Wurth DIN 6325 / ISO 8734 - spina cilindrica temprata diam. 12 mm</t>
+          <t>[CATALOGUE qty0] Wurth DIN 6325 / ISO 8734 - hardened dowel pin diam. 12 mm</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -2188,12 +2188,12 @@
       <c r="M27" s="4" t="n"/>
       <c r="N27" s="3" t="inlineStr">
         <is>
-          <t>Famiglia industriale di spine cilindriche temprate and rettificate, tolleranza m6. La pagina collegata mostra l'esempio diametro 12 x 20 mm; la famiglia offre altre lunghezze.</t>
+          <t>Industrial family of hardened and ground dowel pins, tolerance m6. The linked page shows the diameter 12 x 20 mm example; the family offers other lengths.</t>
         </is>
       </c>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>Catalogo utile al CAD, qty 0. Wurth segnala che DIN 6325 and stata sostituita da DIN EN ISO 8734. Non scegliere 20 mm solo perche and la variante collegata: misurare prima la larghezza dell'assieme and progettare il ritegno.</t>
+          <t>Catalogue useful for the CAD, qty 0. Wurth notes that DIN 6325 has been replaced by DIN EN ISO 8734. Do not choose 20 mm just because it is the linked variant: first measure the width of the assembly and design the retention.</t>
         </is>
       </c>
       <c r="P27" s="4" t="inlineStr">
@@ -2217,7 +2217,7 @@
     <row r="28" hidden="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>[TO SIZE qty0] Ritegni pins and supporti ankle joint</t>
+          <t>[TO SIZE qty0] Pin retainers and supports for the ankle joint</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -2250,12 +2250,12 @@
       <c r="M28" s="4" t="n"/>
       <c r="N28" s="3" t="inlineStr">
         <is>
-          <t>Ritegni smontabili dei due assi di rotazione del giunto foot-shin.</t>
+          <t>Removable retainers for the two rotation axes of the foot-shin joint.</t>
         </is>
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>Ripristinato il catalogo storico: assortimento seeger interni/esterni. Prevedere spallamento stampato o inserto metallico da un lato and ritegno rimovibile dall'altro. Non assumere nut M10, seeger, collare o piastrina prima del CAD: il sistema dipende dal tipo di pin and dalle sedi effettive.</t>
+          <t>Historical catalogue restored: assortment of internal/external circlips. Provide a printed shoulder or metal insert on one side and a removable retainer on the other. Do not assume M10 nut, circlip, collar or plate before the CAD: the system depends on the type of pin and on the actual seats.</t>
         </is>
       </c>
       <c r="P28" s="4" t="inlineStr">
@@ -2279,7 +2279,7 @@
     <row r="29" hidden="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>[SELECTED RITEGNO qty0] Lock nut M10 NERO DIN 985 + Loctite 243 - serra assi Ø12xM10 (ankle + cardano waist)</t>
+          <t>[CHOSEN RETENTION qty0] BLACK M10 self-locking nut DIN 985 + Loctite 243 - clamps the Ø12xM10 axes (ankle + waist gimbal)</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -2312,12 +2312,12 @@
       <c r="M29" s="4" t="n"/>
       <c r="N29" s="3" t="inlineStr">
         <is>
-          <t>Ritegno terminale degli assi rotazione Ø12xM10: il nut M10 serra il filetto della shoulder screw and la rende solidale alle orecchie (4 assi ankle + 2 cardano waist).</t>
+          <t>End retention of the Ø12xM10 rotation axes: the M10 nut clamps the thread of the shoulder screw and makes it integral with the lugs (4 ankle axes + 2 waist gimbal).</t>
         </is>
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>Ritegno SELECTED: nut autobloccante M10 NERO (DIN 985, set nylock M3-M16) + Loctite 243. Expected qty 6 (4 ankle + 2 cardano waist) + scorte; qty 0 fino a CAD. Variante pulita: filettare in un inserto metallico annegato nell'orecchia lontana, cosi il serraggio reagisce su metallo and non comprime il PA-CF.</t>
+          <t>CHOSEN retention: BLACK M10 self-locking nut (DIN 985, nylock set M3-M16) + Loctite 243. Expected qty 6 (4 ankle + 2 waist gimbal) + spares; qty 0 until CAD. Clean variant: thread into a metal insert embedded in the far lug, so that the clamping reacts on metal and does not compress the PA-CF.</t>
         </is>
       </c>
       <c r="P29" s="4" t="inlineStr">
@@ -2403,7 +2403,7 @@
     <row r="31" hidden="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>[CATALOGO qty0] RS PRO 797-6254 - rondella larga M10 DIN 9021 inox, 10.5x30x2.5 mm</t>
+          <t>[CATALOGUE qty0] RS PRO 797-6254 - large washer M10 DIN 9021 stainless steel, 10.5x30x2.5 mm</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -2436,12 +2436,12 @@
       <c r="M31" s="4" t="n"/>
       <c r="N31" s="3" t="inlineStr">
         <is>
-          <t>Rondella larga da valutare sotto testa and nut della vite a spallamento per distribuire il serraggio sulle superfici esterne delle orecchie PA-CF.</t>
+          <t>Large washer to be evaluated under the head and nut of the shoulder screw to distribute the clamping over the outer surfaces of the PA-CF lugs.</t>
         </is>
       </c>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU RS PRO 797-6254: bore 10.5 mm, esterno 30 mm, spessore 2.5 mm, inox A2, DIN 9021. Qty 0: check spazio and quantity dopo CAD. Non usare il serraggio per flettere significativamente le orecchie: il pin and tenuto dal serraggio assiale a quota rated.</t>
+          <t>Exact SKU RS PRO 797-6254: bore 10.5 mm, outer diameter 30 mm, thickness 2.5 mm, stainless steel A2, DIN 9021. Qty 0: verify space and quantity after CAD. Do not use the clamping to significantly bend the lugs: the pin is held by axial clamping at nominal dimension.</t>
         </is>
       </c>
       <c r="P31" s="4" t="inlineStr">
@@ -2465,7 +2465,7 @@
     <row r="32" hidden="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>[CATALOGO qty0] Ruland MSP-12-F - collare split smontabile per pin diam. 12 mm</t>
+          <t>[CATALOGUE qty0] Ruland MSP-12-F - removable split collar for pin diam. 12 mm</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -2498,12 +2498,12 @@
       <c r="M32" s="4" t="n"/>
       <c r="N32" s="3" t="inlineStr">
         <is>
-          <t>Collare in due pcs per ritegno o registro assiale di un pin cilindrico diametro 12 mm quando lo spazio esterno lo consente. Diametro esterno 28 mm, larghezza 11 mm.</t>
+          <t>Two-piece collar for retention or axial adjustment of a 12 mm diameter cylindrical pin when the external space allows it. Outer diameter 28 mm, width 11 mm.</t>
         </is>
       </c>
       <c r="O32" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU MSP-12-F. Price checked 2026-06-02: USD 9.39 about EUR 8.65. Qty 0: and un reference acquistabile, non la scelta automatica; check ingombro esterno and carichi assiali.</t>
+          <t>Exact SKU MSP-12-F. Price verified 2026-06-02: USD 9.39 about EUR 8.65. Qty 0: it is a purchasable reference, not the automatic choice; verify external envelope and axial loads.</t>
         </is>
       </c>
       <c r="P32" s="4" t="inlineStr">
@@ -2655,7 +2655,7 @@
     <row r="35" hidden="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>[ALT qty0] Testa a snodo SKF SA8E M8 destra, bore 8 mm</t>
+          <t>[ALT qty0] SKF SA8E rod end M8 right-hand, bore 8 mm</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -2688,12 +2688,12 @@
       <c r="M35" s="4" t="n"/>
       <c r="N35" s="3" t="inlineStr">
         <is>
-          <t>Upgrade di precisione lato piede.</t>
+          <t>Precision upgrade, foot side.</t>
         </is>
       </c>
       <c r="O35" s="3" t="inlineStr">
         <is>
-          <t>Usare insieme a SAL8E and tubo tenditore.</t>
+          <t>Use together with SAL8E and turnbuckle tube.</t>
         </is>
       </c>
       <c r="P35" s="4" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="36" hidden="1">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>[ALT qty0] Testa a snodo SKF SAL8E M8 sinistra, bore 8 mm</t>
+          <t>[ALT qty0] SKF SAL8E rod end M8 left-hand, bore 8 mm</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -2750,12 +2750,12 @@
       <c r="M36" s="4" t="n"/>
       <c r="N36" s="3" t="inlineStr">
         <is>
-          <t>Upgrade di precisione lato motore.</t>
+          <t>Precision upgrade, motor side.</t>
         </is>
       </c>
       <c r="O36" s="3" t="inlineStr">
         <is>
-          <t>Filetti opposti destra/sinistra per la regolazione.</t>
+          <t>Opposite right/left threads for adjustment.</t>
         </is>
       </c>
       <c r="P36" s="4" t="inlineStr">
@@ -2779,7 +2779,7 @@
     <row r="37" hidden="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>[ALT qty0] Tubo tenditore M8 DIN 1478</t>
+          <t>[ALT qty0] Turnbuckle tube M8 DIN 1478</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -2812,7 +2812,7 @@
       <c r="M37" s="4" t="n"/>
       <c r="N37" s="3" t="inlineStr">
         <is>
-          <t>Corpo del pushrod per upgrade SKF.</t>
+          <t>Pushrod body for the SKF upgrade.</t>
         </is>
       </c>
       <c r="O37" s="3" t="inlineStr"/>
@@ -3093,7 +3093,7 @@
     <row r="42" hidden="1">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>[UPGRADE ROLL qty0] Spaziatori conici high-misalignment M8-&gt;M6 per rod-end metallici (coppia)</t>
+          <t>[ROLL UPGRADE qty0] Conical high-misalignment spacers M8-&gt;M6 for metal rod-ends (pair)</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -3126,12 +3126,12 @@
       <c r="M42" s="4" t="n"/>
       <c r="N42" s="3" t="inlineStr">
         <is>
-          <t>Torque di boccole a gradino/cono: parte cilindrica nel bore Ø8 della sfera, cono stretto verso le orecchie, bullone M6 passante. L'occhio tocca il cono invece della faccia larga -&gt; +8-12 gradi/lato = ±20-25 totali sui rod-end metallici standard.</t>
+          <t>Pair of stepped/conical bushings: cylindrical part in the Ø8 bore of the ball, narrow cone towards the lugs, M6 through bolt. The eye touches the cone instead of the wide face -&gt; +8-12 degrees/side = ±20-25 total on standard metal rod-ends.</t>
         </is>
       </c>
       <c r="O42" s="3" t="inlineStr">
         <is>
-          <t>Alternative economica all'igubal CL per alzare il roll dei rod-end ATTUALI: il pin passa da colletto Ø8 a M6 semplice (meno sezione, ok per ~1-2 kN). Fonti: Competition Supplies 'High misalignment spacer M8 to M6' (coppia, metrico), McGill Motorsport pack 6/10, Midwest Control HMBZC-M8-M6 (USA). Su AliExpress cercare 'heim joint misalignment spacer 8mm'. Qty al CAD.</t>
+          <t>Low-cost alternative to the igubal CL to raise the roll of the CURRENT rod-ends: the pin goes from Ø8 shoulder to plain M6 (less cross-section, ok for ~1-2 kN). Sources: Competition Supplies 'High misalignment spacer M8 to M6' (pair, metric), McGill Motorsport pack 6/10, Midwest Control HMBZC-M8-M6 (USA). On AliExpress search for 'heim joint misalignment spacer 8mm'. Qty at CAD.</t>
         </is>
       </c>
       <c r="P42" s="4" t="inlineStr">
@@ -3279,7 +3279,7 @@
     <row r="45" hidden="1">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>[CATALOGO qty0] Motedis W8H6 - albero precisione diam. 8 mm h6 temprato and rettificato</t>
+          <t>[CATALOGUE qty0] Motedis W8H6 - precision shaft diam. 8 mm h6 hardened and ground</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -3312,12 +3312,12 @@
       <c r="M45" s="4" t="n"/>
       <c r="N45" s="3" t="inlineStr">
         <is>
-          <t>Alternative da tagliare a misura per il pin trasversale piede diametro 8 mm sul quale si montano le due teste a snodo M8.</t>
+          <t>Alternative to be cut to size for the 8 mm diameter foot cross pin on which the two M8 rod ends are mounted.</t>
         </is>
       </c>
       <c r="O45" s="3" t="inlineStr">
         <is>
-          <t>Codice prodotto Motedis W8H6: acciaio CF53 temprato and rettificato, tolleranza h6. Qty 0: prezzo dipendente dalla lunghezza di taglio. Progettare distanziali tra le sfere and ritegni laterali.</t>
+          <t>Motedis product code W8H6: CF53 steel hardened and ground, tolerance h6. Qty 0: price dependent on the cut length. Design spacers between the balls and lateral retainers.</t>
         </is>
       </c>
       <c r="P45" s="4" t="inlineStr">
@@ -3341,7 +3341,7 @@
     <row r="46" hidden="1">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>[CATALOGO qty0] Ruland MSP-8-F - collare split smontabile per pin diam. 8 mm</t>
+          <t>[CATALOGUE qty0] Ruland MSP-8-F - removable split collar for pin diam. 8 mm</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3374,12 +3374,12 @@
       <c r="M46" s="4" t="n"/>
       <c r="N46" s="3" t="inlineStr">
         <is>
-          <t>Collare in due pcs per trattenere lateralmente il pin trasversale piede diametro 8 mm se il CAD lascia spazio. Diametro esterno 18 mm, larghezza 9 mm.</t>
+          <t>Two-piece collar to laterally retain the 8 mm diameter foot cross pin if the CAD leaves space. Outer diameter 18 mm, width 9 mm.</t>
         </is>
       </c>
       <c r="O46" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU MSP-8-F. Price checked 2026-06-02: USD 8.33 about EUR 7.67. Qty 0: valutare due collari oppure un altro ritegno solo dopo aver definito il piede.</t>
+          <t>Exact SKU MSP-8-F. Price verified 2026-06-02: USD 8.33 about EUR 7.67. Qty 0: evaluate two collars or another retainer only after the foot has been defined.</t>
         </is>
       </c>
       <c r="P46" s="4" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="O61" s="7" t="inlineStr">
         <is>
-          <t>G1 mode_11 reference: hip yaw 88 Nm. This is a mostly vertical yaw axis, so gravity torque is near zero and demand is mainly dynamic. RS03 was chosen over RS06 because the estimated aggressive turn at ~45 kg mass was close to the RS06 36 Nm peak limit. ATTENZIONE 2026-07-18: il CAD corrente monta RS06 (36 Nm peak) su hip yaw; questa riga RS03 resta l'intento di acquisto finche' il SIM GATE non decide: log della coppia hip-yaw in curva su Isaac a ~32+ kg; se satura a 36 Nm si ordina RS03 and si adegua il CAD, altrimenti si declassa questa riga a RS06.</t>
+          <t>G1 mode_11 reference: hip yaw 88 Nm. This is a mostly vertical yaw axis, so gravity torque is near zero and demand is mainly dynamic. RS03 was chosen over RS06 because the estimated aggressive turn at ~45 kg mass was close to the RS06 36 Nm peak limit. WARNING 2026-07-18: the current CAD mounts RS06 (36 Nm peak) on hip yaw; this RS03 row remains the purchase intent until the SIM GATE decides: log of the hip-yaw torque while turning in Isaac at ~32+ kg; if it saturates at 36 Nm, RS03 is ordered and the CAD is adapted, otherwise this row is downgraded to RS06.</t>
         </is>
       </c>
       <c r="P61" s="8" t="inlineStr">
@@ -4701,7 +4701,7 @@
     <row r="69" hidden="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>[ALT qty0] RobStride 00 - shoulder pitch/roll alleggerita (2/arm)</t>
+          <t>[ALT qty0] RobStride 00 - lightweight shoulder pitch/roll (2/arm)</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
@@ -4734,12 +4734,12 @@
       <c r="M69" s="4" t="n"/>
       <c r="N69" s="3" t="inlineStr">
         <is>
-          <t>Axes: alternative leggera shoulder pitch/roll. Dimensions: 57 x 57 x 51 mm. Weight: 0.310 kg. Torque RobStride: 5 Nm rated, 14 Nm peak.</t>
+          <t>Axes: lightweight shoulder pitch/roll alternative. Dimensions: 57 x 57 x 51 mm. Weight: 0.310 kg. RobStride torque: 5 Nm rated, 14 Nm peak.</t>
         </is>
       </c>
       <c r="O69" s="3" t="inlineStr">
         <is>
-          <t>Reference G1 mode_11: shoulder pitch/roll 25 Nm per axis. Risparmierebbe 1.244 kg sui quattro giunti ma non puo tenere continuativamente il arm orizzontale with payload 1 kg. Mantenuta solo come alternative per braccia molto leggere and pose intermittenti.</t>
+          <t>G1 mode_11 reference: shoulder pitch/roll 25 Nm per axis. It would save 1.244 kg over the four joints but cannot continuously hold the arm horizontal with a 1 kg payload. Kept only as an alternative for very light arms and intermittent poses.</t>
         </is>
       </c>
       <c r="P69" s="4" t="inlineStr">
@@ -4905,7 +4905,7 @@
     <row r="72" hidden="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>[SECOND CHOICE qty0] RobStride 06 - shoulder yaw piu robusta (1/arm)</t>
+          <t>[SECOND CHOICE qty0] RobStride 06 - sturdier shoulder yaw (1/arm)</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
@@ -4938,12 +4938,12 @@
       <c r="M72" s="4" t="n"/>
       <c r="N72" s="3" t="inlineStr">
         <is>
-          <t>Axis: shoulder yaw, alternative piu robusta. Dimensions: 88 x 88 x 49 mm. Weight: 0.621 kg. Torque RobStride: 11 Nm rated, 36 Nm peak.</t>
+          <t>Axis: shoulder yaw, sturdier alternative. Dimensions: 88 x 88 x 49 mm. Weight: 0.621 kg. RobStride torque: 11 Nm rated, 36 Nm peak.</t>
         </is>
       </c>
       <c r="O72" s="3" t="inlineStr">
         <is>
-          <t>Reference G1 mode_11: shoulder yaw 25 Nm. Riattivare se la shoulder yaw deve muovere carichi a arm esteso o serve piu coppia/rigidita. Salto diretto RS00-&gt;RS06 (RS02 eliminato: dominato, quasi grosso come RS06 ma meta' coppia).</t>
+          <t>G1 mode_11 reference: shoulder yaw 25 Nm. Reactivate if the shoulder yaw has to move loads with the arm extended or more torque/stiffness is needed. Direct jump RS00-&gt;RS06 (RS02 eliminated: dominated, almost as big as RS06 but half the torque).</t>
         </is>
       </c>
       <c r="P72" s="4" t="inlineStr">
@@ -5245,7 +5245,7 @@
     <row r="77" hidden="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>[SECOND CHOICE qty0] RobStride 06 - wrist 3 assi (riserva piu robusta)</t>
+          <t>[SECOND CHOICE qty0] RobStride 06 - 3-axis wrist (sturdier reserve)</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -5278,12 +5278,12 @@
       <c r="M77" s="4" t="n"/>
       <c r="N77" s="3" t="inlineStr">
         <is>
-          <t>Riserva robusta per i 3 assi del wrist. Dimensions: 88 x 88 x 49 mm. Weight: 0.621 kg. Torque RobStride: 11 Nm rated, 36 Nm peak.</t>
+          <t>Sturdy reserve for the 3 wrist axes. Dimensions: 88 x 88 x 49 mm. Weight: 0.621 kg. RobStride torque: 11 Nm rated, 36 Nm peak.</t>
         </is>
       </c>
       <c r="O77" s="3" t="inlineStr">
         <is>
-          <t>Reference G1 mode_11: wrist roll 25 Nm, pitch/yaw 5 Nm. Riserva se servisse molta piu coppia/rigidita al wrist; salto RS00-&gt;RS06 (RS02 eliminato perche' dominato). Per il wrist RS00 resta ampiamente sufficiente.</t>
+          <t>G1 mode_11 reference: wrist roll 25 Nm, pitch/yaw 5 Nm. Reserve in case much more torque/stiffness were needed at the wrist; jump RS00-&gt;RS06 (RS02 eliminated because dominated). For the wrist RS00 remains amply sufficient.</t>
         </is>
       </c>
       <c r="P77" s="4" t="inlineStr">
@@ -5449,7 +5449,7 @@
     <row r="80" hidden="1">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>[SECOND CHOICE qty0] RobStride 05 - wrist pitch/yaw ultraleggero (2/arm)</t>
+          <t>[SECOND CHOICE qty0] RobStride 05 - ultralight wrist pitch/yaw (2/arm)</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -5482,12 +5482,12 @@
       <c r="M80" s="4" t="n"/>
       <c r="N80" s="3" t="inlineStr">
         <is>
-          <t>Axes: wrist pitch/yaw, alternative ultraleggera. Dimensions: 46 x 46 x 44 mm. Weight: 0.191 kg. Torque RobStride: 1.6 Nm rated, 5.5 Nm peak.</t>
+          <t>Axes: wrist pitch/yaw, ultralight alternative. Dimensions: 46 x 46 x 44 mm. Weight: 0.191 kg. RobStride torque: 1.6 Nm rated, 5.5 Nm peak.</t>
         </is>
       </c>
       <c r="O80" s="3" t="inlineStr">
         <is>
-          <t>Reference G1 mode_11: wrist pitch/yaw 5 Nm: RS05 (5.5 peak) and la taglia esatta and pesa solo 0.191 kg. Alternative all'RS00 SE il payload in mano resta &lt;1 kg: rated 1.6 Nm limita il carico continuo. Piu leggera ma meno robusta and without il margine dell'RS00.</t>
+          <t>G1 mode_11 reference: wrist pitch/yaw 5 Nm: RS05 (5.5 peak) is the exact size and weighs only 0.191 kg. Alternative to the RS00 IF the payload in the hand stays &lt;1 kg: rated 1.6 Nm limits the continuous load. Lighter but less sturdy and without the margin of the RS00.</t>
         </is>
       </c>
       <c r="P80" s="4" t="inlineStr">
@@ -7448,7 +7448,7 @@
     <row r="112" hidden="1">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>[TO DESIGN qty0] Cover isolante ventilata per PDU, fusibili and condensatori</t>
+          <t>[TO DESIGN qty0] Ventilated insulating cover for PDU, fuses and capacitors</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
@@ -7486,7 +7486,7 @@
       </c>
       <c r="O112" s="3" t="inlineStr">
         <is>
-          <t>Obbligatorio prima del collaudo completo. Disegnarlo dopo il layout del pannello elettrico; lasciare accesso manutenzione and ventilazione al Regen Clamp and alla sua resistenza, che devono essere montati su alluminio.</t>
+          <t>Mandatory before full commissioning tests. Design it after the electrical panel layout; leave maintenance access and ventilation for the Regen Clamp and its resistor, which must be mounted on aluminium.</t>
         </is>
       </c>
       <c r="P112" s="4" t="inlineStr">
@@ -8696,12 +8696,12 @@
       <c r="M132" s="4" t="n"/>
       <c r="N132" s="3" t="inlineStr">
         <is>
-          <t>Sezionatore manuale di bordo sul positivo battery per manutenzione and distacco fisico di emergenza. Non sostituisce il contattore automatico SW80B-10 ne il fungo XB5AS8442. Riserva CAD prudente 70 x 70 x 100 mm incluso spazio maniglia; massa BOM 0.468 kg.</t>
+          <t>On-board manual disconnect switch on the battery positive for maintenance and emergency physical disconnection. It does not replace the SW80B-10 automatic contactor nor the XB5AS8442 mushroom button. Prudent CAD reserve 70 x 70 x 100 mm including handle space; BOM mass 0.468 kg.</t>
         </is>
       </c>
       <c r="O132" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU ED250B-1. Price checked 2026-06-02: EUR 91 netto / EUR 109.20 IVA inclusa. Rating 250 A continui, 96 VDC with blowouts. Usarlo come sezionatore a vuoto o emergenza, non come interruttore ordinario sotto carico; check la sagoma definitiva dal disegno Albright prima dei fori.</t>
+          <t>Exact SKU ED250B-1. Price verified 2026-06-02: EUR 91 net (excluding VAT) / EUR 109.20 VAT included. Rating 250 A continuous, 96 VDC with blowouts. Use it as a no-load or emergency disconnect switch, not as an ordinary switch under load; verify the final outline from the Albright drawing before making the holes.</t>
         </is>
       </c>
       <c r="P132" s="4" t="inlineStr">
@@ -8853,7 +8853,7 @@
     <row r="135" hidden="1">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>[ALT qty0] Dan-Tech Energy Softpack 13S5P 48V 25Ah 100A - configurare Smart BMS + AS150U</t>
+          <t>[ALT qty0] Dan-Tech Energy Softpack 13S5P 48V 25Ah 100A - configure Smart BMS + AS150U</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
@@ -8886,12 +8886,12 @@
       <c r="M135" s="4" t="n"/>
       <c r="N135" s="3" t="inlineStr">
         <is>
-          <t>Alternative pronta in formato minimale termoretraibile: 65 celle cilindriche Samsung INR21700-50S, 1200 Wh, 100 A continui, 200 A peak, 280 x 80 x 130 mm, 5.2 kg.</t>
+          <t>Ready-made alternative in minimal heat-shrink format: 65 Samsung INR21700-50S cylindrical cells, 1200 Wh, 100 A continuous, 200 A peak, 280 x 80 x 130 mm, 5.2 kg.</t>
         </is>
       </c>
       <c r="O135" s="3" t="inlineStr">
         <is>
-          <t>Pagina prodotto esatta. Prezzo visibile 2026-06-02: EUR 741 IVA inclusa per configurazione base XT90 without BMS; prima dell'ordine chiedere il totale della variante Smart BMS + AS150U. Non attivare la riga without BMS.</t>
+          <t>Exact product page. Price visible 2026-06-02: EUR 741 VAT included for the base XT90 configuration without BMS; before ordering ask for the total of the Smart BMS + AS150U variant. Do not activate the row without BMS.</t>
         </is>
       </c>
       <c r="P135" s="4" t="inlineStr">
@@ -9742,7 +9742,7 @@
     <row r="150" hidden="1">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>[OPZIONE qty0] Computer low-level realtime separato per locomozione</t>
+          <t>[OPTION qty0] Separate low-level realtime computer for locomotion</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
@@ -9775,12 +9775,12 @@
       <c r="M150" s="4" t="n"/>
       <c r="N150" s="3" t="inlineStr">
         <is>
-          <t>Supervisore deterministico tra policy and attuatori: legge IMU and feedback giunti, invia setpoint RobStride sui bus CAN, applica limiti, heartbeat, watchdog and transizione sicura in damping/stop. Non sostituisce i loop interni dei motors.</t>
+          <t>Deterministic supervisor between policy and actuators: reads IMU and joint feedback, sends RobStride setpoints on the CAN buses, applies limits, heartbeat, watchdog and safe transition to damping/stop. It does not replace the internal loops of the motors.</t>
         </is>
       </c>
       <c r="O150" s="3" t="inlineStr">
         <is>
-          <t>Non comprare inizialmente: baseline prototipo Thor-only with processo realtime isolato, SocketCAN diretto and safety hardware indipendente. Valutare controller separato solo se i test mostrano jitter, saturazione/interfacce CAN insufficienti oppure se serve isolamento dai crash del software AI. Non scegliere Raspberry Pi, MCU o SBC prima di aver misurato frequenza loop, latenza and jitter.</t>
+          <t>Do not buy initially: Thor-only prototype baseline with isolated realtime process, direct SocketCAN and independent hardware safety. Evaluate a separate controller only if tests show jitter, saturation/insufficient CAN interfaces, or if isolation from crashes of the AI software is needed. Do not choose Raspberry Pi, MCU or SBC before having measured loop frequency, latency and jitter.</t>
         </is>
       </c>
       <c r="P150" s="4" t="inlineStr">
@@ -10312,7 +10312,7 @@
     <row r="159" hidden="1">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>[TO DESIGN qty0] Harness custom RS03/RS04: XT30UW-F + GH1.25 CAN + strain relief</t>
+          <t>[TO DESIGN qty0] Custom harness RS03/RS04: XT30UW-F + GH1.25 CAN + strain relief</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
@@ -10345,12 +10345,12 @@
       <c r="M159" s="4" t="n"/>
       <c r="N159" s="3" t="inlineStr">
         <is>
-          <t>Fascio da costruire dopo il CAD per RS04 gambe, RS03 hip yaw and RS03 waist roll. Usa i connettori acquistabili elencati sopra, cavo potenza dimensionato and doppino CAN.</t>
+          <t>Harness to be built after the CAD for RS04 legs, RS03 hip yaw and RS03 waist roll. It uses the purchasable connectors listed above, sized power cable and CAN twisted pair.</t>
         </is>
       </c>
       <c r="O159" s="3" t="inlineStr">
         <is>
-          <t>Non esiste un link a un harness completo RobStride per questo umanoide. Il manuale RS04 definisce i terminali lato cavo; K-Scale conferma che il wiring richiede progettazione and strain relief. Per i microcontatti JST GH commissionare preferibilmente crimpatura and collaudo a un cablatore: la pinza ufficiale JST YRS-1590 and elencata come opzione qty 0 ma costa molto. Questa riga resta qty 0 per evitare un costo fittizio.</t>
+          <t>There is no link to a complete RobStride harness for this humanoid. The RS04 manual defines the cable-side terminals; K-Scale confirms that the wiring requires design and strain relief. For the JST GH micro-contacts, preferably commission crimping and testing to a cable assembler: the official JST YRS-1590 crimping tool is listed as a qty 0 option but is very expensive. This row stays qty 0 to avoid a fictitious cost.</t>
         </is>
       </c>
       <c r="P159" s="4" t="inlineStr">
@@ -10374,7 +10374,7 @@
     <row r="160" hidden="1">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>[TO DESIGN qty0] Wiring Thor J47 -&gt; CANH/CANL per 2 bus nativi</t>
+          <t>[TO DESIGN qty0] Wiring Thor J47 -&gt; CANH/CANL for 2 native buses</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
@@ -10407,12 +10407,12 @@
       <c r="M160" s="4" t="n"/>
       <c r="N160" s="3" t="inlineStr">
         <is>
-          <t>Wiring dal connettore J47 del dev kit Thor ai due bus delle gambe. Il dev kit espone fisicamente CANH and CANL: non serve uno SN65HVD230 esterno.</t>
+          <t>Wiring from the J47 connector of the Thor dev kit to the two leg buses. The dev kit physically exposes CANH and CANL: an external SN65HVD230 is not needed.</t>
         </is>
       </c>
       <c r="O160" s="3" t="inlineStr">
         <is>
-          <t>Il mating connector and il pinout del wiring vanno verificati sulla documentazione Thor and sul kit fisico prima dell'acquisto. Riga qty 0: non inventare uno SKU.</t>
+          <t>The mating connector and the pinout of the wiring must be verified against the Thor documentation and the physical kit before purchase. Qty 0 row: do not invent an SKU.</t>
         </is>
       </c>
       <c r="P160" s="4" t="inlineStr">
@@ -11043,12 +11043,12 @@
       <c r="M170" s="4" t="n"/>
       <c r="N170" s="3" t="inlineStr">
         <is>
-          <t>Capicorda per i due terminali M10 del sezionatore ED250B-1 sul tronco positivo da 25 mm2. Due pcs installati and due di scorta.</t>
+          <t>Cable lugs for the two M10 terminals of the ED250B-1 disconnect switch on the 25 mm2 positive trunk. Two pieces installed and two spare.</t>
         </is>
       </c>
       <c r="O170" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU Klauke 704F10. Progettato per conduttori fini and superfini classe 5 and 6, rame EN13600 stagnato. Price checked 2026-06-02: GBP 1.75 netto each about EUR 2.10.</t>
+          <t>Exact SKU Klauke 704F10. Designed for fine and extra-fine stranded conductors class 5 and 6, tinned EN13600 copper. Price verified 2026-06-02: GBP 1.75 net (excluding VAT) each about EUR 2.10.</t>
         </is>
       </c>
       <c r="P170" s="4" t="inlineStr">
@@ -11320,7 +11320,7 @@
     <row r="175" hidden="1">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>[OPZIONE qty0] JST YRS-1590 - pinza ufficiale per contatti GH SSHL-002T-P0.2</t>
+          <t>[OPTION qty0] JST YRS-1590 - official crimping tool for GH contacts SSHL-002T-P0.2</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
@@ -11353,12 +11353,12 @@
       <c r="M175" s="4" t="n"/>
       <c r="N175" s="3" t="inlineStr">
         <is>
-          <t>Pinza ufficiale per crimpare i microcontatti JST GH dei fasci CAN RS03/RS04. Non serve se il cablatore fornisce i fasci gia assemblati and collaudati.</t>
+          <t>Official tool for crimping the JST GH micro-contacts of the RS03/RS04 CAN harnesses. Not needed if the cable assembler supplies the harnesses already assembled and tested.</t>
         </is>
       </c>
       <c r="O175" s="3" t="inlineStr">
         <is>
-          <t>Exact SKU JST YRS-1590. DigiKey indicava USD 1736.95 about EUR 1595 il 2026-06-02. Per quindici motors and normalmente piu sensato commissionare i fasci a un cablatore and richiedere prova di trazione and test continuita, invece di comprare la pinza.</t>
+          <t>Exact SKU JST YRS-1590. DigiKey indicated USD 1736.95 about EUR 1595 on 2026-06-02. For fifteen motors it is normally more sensible to commission the harnesses to a cable assembler and request a pull test and continuity test, instead of buying the tool.</t>
         </is>
       </c>
       <c r="P175" s="4" t="inlineStr">
@@ -12853,7 +12853,7 @@
     <row r="202" hidden="1">
       <c r="A202" s="3" t="inlineStr">
         <is>
-          <t>[REF qty0] Unitree G1 mode_11 URDF ufficiale</t>
+          <t>[REF qty0] Unitree G1 mode_11 official URDF</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
@@ -12886,12 +12886,12 @@
       <c r="M202" s="4" t="n"/>
       <c r="N202" s="3" t="inlineStr">
         <is>
-          <t>Baseline geometrica and limiti per axis del G1 29 DOF corrente.</t>
+          <t>Geometric baseline and per-axis limits of the current G1 29 DOF.</t>
         </is>
       </c>
       <c r="O202" s="3" t="inlineStr">
         <is>
-          <t>Usare origini giunti and mesh come reference. L'URDF descrive la cinematica virtuale, non espone il CAD interno del leveraggio ankle.</t>
+          <t>Use joint origins and meshes as a reference. The URDF describes the virtual kinematics; it does not expose the internal CAD of the ankle linkage.</t>
         </is>
       </c>
       <c r="P202" s="4" t="inlineStr">
@@ -12915,7 +12915,7 @@
     <row r="203" hidden="1">
       <c r="A203" s="3" t="inlineStr">
         <is>
-          <t>[REF qty0] Unitree G1 description README ufficiale</t>
+          <t>[REF qty0] Unitree G1 description official README</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
@@ -12948,12 +12948,12 @@
       <c r="M203" s="4" t="n"/>
       <c r="N203" s="3" t="inlineStr">
         <is>
-          <t>Elenco modelli G1 and stato aggiornato/deprecato.</t>
+          <t>List of G1 models and updated/deprecated status.</t>
         </is>
       </c>
       <c r="O203" s="3" t="inlineStr">
         <is>
-          <t>mode_11 and la baseline 29 DOF non bloccata and aggiornata.</t>
+          <t>mode_11 is the unlocked and up-to-date 29 DOF baseline.</t>
         </is>
       </c>
       <c r="P203" s="4" t="inlineStr">
@@ -12977,7 +12977,7 @@
     <row r="204" hidden="1">
       <c r="A204" s="3" t="inlineStr">
         <is>
-          <t>[REF qty0] Unitree G1-Comp pagina ufficiale - testa 2 DOF</t>
+          <t>[REF qty0] Unitree G1-Comp official page - 2 DOF head</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
@@ -13010,12 +13010,12 @@
       <c r="M204" s="4" t="n"/>
       <c r="N204" s="3" t="inlineStr">
         <is>
-          <t>Reference ufficiale per aggiungere due motors neck.</t>
+          <t>Official reference for adding two neck motors.</t>
         </is>
       </c>
       <c r="O204" s="3" t="inlineStr">
         <is>
-          <t>La pagina dichiara Head 2 degrees of freedom = 2, ma non pubblica la coppia dei due motors.</t>
+          <t>The page states Head 2 degrees of freedom = 2, but does not publish the torque of the two motors.</t>
         </is>
       </c>
       <c r="P204" s="4" t="inlineStr">
@@ -13039,7 +13039,7 @@
     <row r="205" hidden="1">
       <c r="A205" s="3" t="inlineStr">
         <is>
-          <t>[REF qty0] Unitree G1-EDU Waist Fastener manuale ufficiale</t>
+          <t>[REF qty0] Unitree G1-EDU Waist Fastener official manual</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
@@ -13072,12 +13072,12 @@
       <c r="M205" s="4" t="n"/>
       <c r="N205" s="3" t="inlineStr">
         <is>
-          <t>Reference ufficiale per la waist opzionale G1 EDU sbloccabile and bloccabile.</t>
+          <t>Official reference for the optional G1 EDU waist that can be unlocked and locked.</t>
         </is>
       </c>
       <c r="O205" s="3" t="inlineStr">
         <is>
-          <t>Conferma la waist articolata opzionale; il dettaglio interno del leveraggio va ricostruito in CAD.</t>
+          <t>Confirms the optional articulated waist; the internal detail of the linkage has to be reconstructed in CAD.</t>
         </is>
       </c>
       <c r="P205" s="4" t="inlineStr">
@@ -13134,12 +13134,12 @@
       <c r="M206" s="4" t="n"/>
       <c r="N206" s="3" t="inlineStr">
         <is>
-          <t>Reference open hardware da tenere sotto osservazione.</t>
+          <t>Open hardware reference to keep under observation.</t>
         </is>
       </c>
       <c r="O206" s="3" t="inlineStr">
         <is>
-          <t>K-Bot usa solo RobStride ma ha 20 DOF and una ankle diretta a un axis: non copiare la sua ankle per la baseline G1.</t>
+          <t>K-Bot uses only RobStride but has 20 DOF and a direct single-axis ankle: do not copy its ankle for the G1 baseline.</t>
         </is>
       </c>
       <c r="P206" s="4" t="inlineStr">

</xml_diff>